<commit_message>
Final changes done by adding new features and cleaning the code
</commit_message>
<xml_diff>
--- a/linkedin_posts.xlsx
+++ b/linkedin_posts.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,25 +429,30 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Model Expectation</t>
+          <t>User Expectation</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Final LinkedIn Post</t>
+          <t>Processing Workflow</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Final LinkedIn Post / Reason</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Tokens In</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Tokens Out</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -466,24 +471,35 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>**Rethink Work, Reimagine Growth** 🤖💻 As automation, remote collaboration, and AI-driven decision-making reshape the future of work, organizations must adapt and lead the change. The Challenge: outdated team structures, underdeveloped skills, and unproductive human-machine collaboration.
-The Change: invest in upskilling, reskill, and adopt a hybrid work model that leverages AI and human capabilities. This will enable teams to work smarter, not harder, and drive innovation and growth.
-The Outcome: a future-proof workforce that is agile, adaptable, and equipped to thrive in a world where machines and humans collaborate productively.
-What steps is your organization taking to future-proof your workforce and drive growth in the age of automation and AI?</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>**The future of work is evolving faster than ever!** 🌍💼
+Automation, remote collaboration, and AI-driven decision-making are transforming the workplace as we know it. 
+🚀 Challenge: Traditional team structures and skill development methods are struggling to keep pace with these changes.
+🔄 Change: Forward-thinking organizations are reimagining:
+- How they structure teams to adapt to shifting dynamics
+- How they upskill and reskill their workforce to stay competitive
+- How humans and machines can collaborate seamlessly to maximize productivity
+✅ Outcome: Those who embrace this shift are not only keeping up but leading the charge into a more innovative and efficient future.
+How is your organization preparing for the future of work? I'd love to hear your thoughts and strategies! 👇
+#FutureOfWork #Automation #AI #RemoteWork #Upskilling #Collaboration #WorkplaceInnovation</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>43</v>
       </c>
-      <c r="F2" t="n">
-        <v>152</v>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="n">
+        <v>176</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -492,7 +508,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>India became the world’s largest economy in 2025, surpassing the United States and China. This shift dramatically altered global trade flows, political alliances, and economic power structures across continents.</t>
+          <t>India became the world's largest economy in 2025, surpassing the United States and China. This shift dramatically altered global trade flows, political alliances, and economic power structures across continents.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -502,29 +518,36 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FACT_CHECK_AND_GENERATE</t>
+          <t>The system will verify the factual claim using external sources. If verified, the output will reference validated facts and may include contextual explanation, implications, or informed recommendations. If not verified, corrective information will be provided instead of a post.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Are we ready for a new world order? 🌎 **India's historic leap to the world's largest economy has just begun**. With its GDP surpassing the United States and China, a seismic shift is unfolding that will reshape global trade, politics, and economic power dynamics for generations to come.
-This monumental change will challenge the long-standing status quo and create new opportunities for growth, innovation, and collaboration. As the world grapples with the implications of this shift, businesses, policymakers, and individuals must adapt and evolve to thrive in this new landscape.
-Key takeaways from this transformation include:
-*   A new era of economic cooperation and competition is emerging, with India at the forefront
-*   Traditional trade routes and supply chains will need to be reassessed and reimagined
-*   The balance of global power is shifting, with far-reaching consequences for international relations and economic policy
-What skills and strategies will you need to succeed in this new world order? 🤔💼 #IndiasRise #GlobalEconomy #NewWorldOrder #EconomicShift #GDP #Trade #Politics #PowerDynamics</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>38</v>
+          <t>User Input → Intent Classification → Safety Validation → Search Query Generation → External Fact Retrieval → Fact Verification → Reference-Aware Content Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VERDICT: false
+VERIFIED FACTS:
+- India became the world's fourth-largest economy in 2025, surpassing Japan.
+- India is projected to become the third-largest economy within the next few years, but it has not surpassed the United States or China.
+CORRECTION (if false):
+India did not become the world's largest economy in 2025. It ranked fourth globally, behind the United States, China, and Germany, according to nominal GDP rankings.
+EVIDENCE URLS:
+- https://www.dw.com/en/india-overtakes-japan-as-4th-largest-economy-report-says/a-75341063  
+- https://statisticstimes.com/economy/projected-world-gdp-ranking.php  </t>
+        </is>
       </c>
       <c r="F3" t="n">
-        <v>220</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
+        <v>37</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>FACT_REJECTED</t>
         </is>
       </c>
     </row>
@@ -541,17 +564,26 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="n">
-        <v>0</v>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>I'm sorry, but I cannot assist with this topic. Please consider discussing lawful and ethical approaches to workplace management.</t>
+        </is>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
@@ -570,28 +602,32 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>**Execution Over Excitement: Why Startups Fail** 💡
-Many startups fail not because of bad ideas, but due to poor execution, lack of market understanding, and inability to adapt to customer feedback and changing business conditions.
-In today's fast-paced startup landscape, having a great idea is just the starting point. What sets successful startups apart is their ability to execute, adjust, and innovate in response to market needs.
-Here are three key takeaways to avoid the startup pitfalls:
-- Develop a deep understanding of your target market and customer needs.
-- Build a strong team that can adapt quickly to changing business conditions.
-- Foster a culture of continuous learning and improvement.
-Can you share your experience with startup execution and how you overcame common challenges?</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>**Why do so many startups fail?** 💡
+The challenge: Startups often begin with brilliant ideas but stumble in execution. 
+The change: Success isn’t just about having a groundbreaking concept—it’s about understanding the market, listening to customer feedback, and adapting to ever-changing business conditions. 
+The outcome: Companies that master these elements are far more likely to thrive in competitive landscapes, while those that don’t risk falling behind.
+Execution, adaptability, and customer-centricity are the true pillars of sustainable startup success. 
+What do you think is the most critical factor for a startup's success? 🧐
+#Startups #Entrepreneurship #BusinessGrowth #CustomerFeedback #Adaptability #Execution #Innovation</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>32</v>
       </c>
-      <c r="F5" t="n">
-        <v>149</v>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="n">
+        <v>144</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -610,42 +646,36 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>VERDICT: true
-VERIFIED FACTS:
-- Artificial intelligence in healthcare can assist doctors in diagnostics, patient monitoring, and treatment planning.
-- Ethical concerns like data privacy, bias, and accountability still remain unresolved in AI-assisted healthcare.
-CORRECTION: None
-EVIDENCE URLS:
-- https://www.ualberta.ca/en/law/media-library/faculty-research/hli/research/docs/privacy-concerns-with-commercial-artificial-intelligence-for-healthcare.pdf
-- https://www.tonic.ai/guides/ai-healthcare-data-privacy-ethics
-- https://healthtechmagazine.net/article/2024/10/addressing-trust-and-privacy-concerns-support-full-scale-ai-adoption-healthcare
-- https://www.jimersonfirm.com/blog/2026/02/healthcare-ai-regulation-2025-new-compliance-requirements-every-provider-must-know/
-- https://www.nature.com/articles/s41746-023-00858-z
-- https://www.nature.com/articles/s41591-021-01595-0
-- https://pmc.ncbi.nlm.nih.gov/articles/PMC11542778/
-- https://www.jyi.org/2026-january-1/2026/1/8/bias-in-medical-ai-algorithmic-fairness-and-ethics-challenges
-- https://www.futuremedicine.com/articles/ai-bias-a-problem-long-before-the-algorithm
-- https://royalsocietypublishing.org/rsos/article/12/5/241873/235732/Ethical-and-legal-considerations-in-healthcare-AI
-- https://www.ama-assn.org/practice-management/digital-health/implement-health-ai-first-decide-who-s-accountable
-- https://www.sciencedirect.com/science/article/pii/S2772501422000185
-- https://www.fsmb.org/siteassets/advocacy/policies/incorporation-of-ai-into-practice.pdf
-- https://www.sciencedirect.com/science/article/pii/S1078817425000926</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>**Can AI revolutionize healthcare while addressing its ethical dilemmas?** 🤔
+Artificial intelligence is making waves in healthcare. From enhancing diagnostics to streamlining patient monitoring and treatment planning, the potential is immense. 🚀
+Yet, challenges remain:
+- **Data Privacy:** How do we ensure sensitive patient data is protected?
+- **Bias in Algorithms:** Can we eliminate prejudices embedded in the systems?
+- **Accountability:** Who takes responsibility when AI makes a critical error?
+The promise of AI in healthcare is exciting, but addressing these ethical concerns is crucial for its responsible adoption.
+🔍 What are your thoughts on balancing innovation with ethics in AI-driven healthcare? 
+#ArtificialIntelligence #HealthcareInnovation #EthicsInAI #DataPrivacy #FutureOfHealthcare #AI</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>32</v>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>FACT_REJECTED</t>
+      <c r="G6" t="n">
+        <v>155</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -662,29 +692,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>**Climate Crisis: The Time for Action is Now** 🌎💧
-As a global community, we're faced with a stark reality: climate change is no longer a looming threat, but a present-day crisis that's ravaging our agriculture, draining our water resources, and straining our urban infrastructure. The urgent question is: what can we do to stem the tide of this catastrophe?
-The challenge is clear: we must take collective action to mitigate the effects of climate change. This requires governments and individuals to work together, leveraging their unique strengths and expertise to develop and implement effective solutions. By doing so, we can create a more resilient and sustainable future for all.
-Here are three key steps to get us started:
-• Invest in renewable energy sources and green infrastructure
-• Implement sustainable land use practices and reforestation efforts
-• Enhance climate-resilient agriculture and water management systems
-So, what role will you play in the fight against climate change? 💚
-#Sustainability #ClimateAction #EnvironmentalLeadership #RenewableEnergy #SustainableLiving</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>**Climate change is no longer a future threat—it’s a present reality. 🌍**
+The impacts are clear and undeniable. Agriculture is under strain, water resources are depleting, and urban infrastructure is being tested like never before. 
+It’s no longer about predicting the future—it’s about addressing the challenges we face today.
+- How can we build sustainable agricultural systems to withstand these changes?
+- What steps can be taken to safeguard water resources?
+- How do we make urban infrastructure more resilient?
+Governments, organizations, and individuals must come together in coordinated action to mitigate these effects and secure a livable future. 
+**What innovations or strategies do you think can help tackle these challenges effectively?** 💡
+#ClimateChange #Sustainability #UrbanPlanning #WaterResources #Agriculture #EnvironmentalAction #Resilience</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>34</v>
       </c>
-      <c r="F7" t="n">
-        <v>212</v>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="n">
+        <v>166</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -703,27 +738,33 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>**Financial Literacy for the Future: Why Early Education Matters** 📚💸
-Financial literacy is no longer a nicety, but a necessity in today's complex economic landscape. Research shows that individuals who understand basic financial concepts are more likely to achieve long-term financial stability and success.
-**The Challenge:** Many adults struggle with managing savings, investments, and debt due to a lack of financial education. This can lead to financial stress, decreased savings rates, and reduced financial security.
-**The Change:** By incorporating financial literacy into early education, we can empower future generations with the knowledge and skills needed to navigate the financial world with confidence.
-**The Outcome:** Early financial education can lead to better financial decision-making, increased savings rates, and improved long-term financial planning. It's time to prioritize financial literacy in our schools and communities.
-What steps can we take to make financial literacy a priority in our education system? 🤔
-#FinancialLiteracy #EarlyEducation #FinancialStability #EconomicSecurity #FinancialPlanning</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>**When should financial literacy start? As early as possible. 💡**
+In today’s complex economic environment, managing savings, investments, debt, and long-term financial planning has become more critical than ever. Yet, many of us enter adulthood without the foundational knowledge needed to navigate these challenges effectively.
+**The Challenge:** Lack of financial education early in life leaves many struggling with poor financial decisions later on.
+**The Change:** Incorporating financial literacy into early education can empower individuals with the tools to make informed choices.
+**The Outcome:** A generation better equipped to handle their finances, leading to reduced debt, smarter investments, and greater financial stability.
+Let’s prioritize financial education and give young minds the knowledge they need to thrive. 📚
+**What’s your take? Should financial literacy be a mandatory part of the school curriculum?**
+#FinancialLiteracy #EducationMatters #PersonalFinance #FinancialPlanning #InvestSmart #EconomicAwareness #FutureReady</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>31</v>
       </c>
-      <c r="F8" t="n">
-        <v>200</v>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="n">
+        <v>190</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -742,29 +783,33 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">**The Future of Education: Are We Ready to Think Differently?** 🤔💡
-As we navigate an increasingly complex world, it's clear that traditional education systems need a significant overhaul. Rote learning and memorization are no longer sufficient to equip students with the skills they need to succeed. Instead, we must focus on cultivating critical thinking, creativity, and problem-solving abilities that will serve them well in the real world.
-The challenge is clear: how can we transform our education systems to prioritize these essential skills?
-Here are three key areas of focus:
- • **Integrate project-based learning** to encourage students to apply theoretical knowledge to real-world problems.
- • **Foster collaboration and communication skills** to prepare students for the diverse, global communities they'll encounter in their careers.
- • **Emphasize experimentation and failure** to teach students the value of taking calculated risks and learning from their mistakes.
-So, what steps can we take to revolutionize education and give students the skills they need to thrive in the 21st century?
-</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>**Are we preparing students for the future or the past?** 🌍📚  
+The education system has long relied on rote learning—memorizing facts and repeating them during exams. But does this truly equip students for real-world challenges?  
+🔄 Challenge: Students often graduate with theoretical knowledge but lack critical thinking, creativity, and problem-solving skills.  
+✨ Change: Shifting the focus from rote memorization to fostering curiosity and innovation in classrooms.  
+✅ Outcome: A generation better equipped to address complex, real-world problems with confidence and adaptability.  
+It's time to reimagine education to align with the demands of a rapidly evolving world.  
+**How can schools integrate critical thinking and creativity into their curriculums?** Share your ideas below!  
+#EducationReform #CriticalThinking #Creativity #ProblemSolving #FutureSkills #LifelongLearning #InnovationInEducation</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
         <v>29</v>
       </c>
-      <c r="F9" t="n">
-        <v>207</v>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" t="n">
+        <v>179</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -783,17 +828,26 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BLOCK_CONTENT</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="n">
-        <v>0</v>
+          <t>The system will block the request and will not generate any content. A brief explanation will be returned without recommendations or references.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Hate Speech Detection → Content Blocked</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>I'm sorry, but this topic is not appropriate for a LinkedIn post as it promotes a discriminatory perspective. Please consider discussing a more inclusive or constructive topic.</t>
+        </is>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
@@ -812,38 +866,34 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Invalid json output: {
-  "formatted_post": "**The Double-Edged Sword of Social Media: Amplifying Voices and Challenges** 💻💬\
-  The rapid proliferation of social media has brought about a profound shift in the way we communicate. On one hand, it has empowered individuals to amplify their voices, share their perspectives, and connect with others across the globe. On the other hand, it has also contributed to the spread of misinformation, reduced attention spans, and exacerbated mental health challenges.\
-  As we navigate this complex digital landscape, it's essential to acknowledge both the benefits and drawbacks of social media.\
-  • Increased connectivity and global awareness\
-  • Easier access to information and resources\
-  • Amplified voices for marginalized communities\
-  • Misinformation and disinformation spread quickly\
-  • Reduced attention spans and decreased focus\
-  • Mental health challenges and increased stress\
-  How can we harness the power of social media to create a more balanced and healthy online environment?",
-  "need_references": false,
-  "reference_queries": [],
-  "recommendations": []
-}
-For troubleshooting, visit: https://docs.langchain.com/oss/python/langchain/errors/OUTPUT_PARSING_FAILURE </t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>**How has social media shaped our communication—for better or worse?** 🌐
+Social media revolutionized how we connect, share, and amplify voices. But it hasn’t been without its challenges. 
+**The Challenge:** The rise of platforms made information accessible like never before, but also introduced issues like misinformation, reduced attention spans, and mental health concerns.
+**The Change:** As users, industries, and governments begin to recognize these impacts, efforts to promote digital literacy, fact-checking, and mindful usage are gaining traction.
+**The Outcome:** Balancing the benefits of connectivity with the risks of misuse is key. Social media can empower communities and individuals, but it requires conscious effort to use it responsibly.
+What strategies do you think can help us harness the positives while minimizing the downsides? 💬
+#SocialMedia #Communication #DigitalTransformation #MentalHealth #Misinformation #OnlineBehavior</t>
+        </is>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+        <v>29</v>
+      </c>
+      <c r="G11" t="n">
+        <v>180</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -860,31 +910,35 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>**Break Free from Competition: How Small Businesses Can Level Up with Digital Marketing** 🚀💻
-Are you tired of feeling like your small business is getting lost in the noise? The good news is that you don't have to compete on the same level as larger corporations. By leveraging digital marketing, online platforms, and data analytics, you can reach a global audience more effectively and take your business to the next level.
-Challenge: Limited resources and budget constraints make it difficult for small businesses to compete with larger corporations.
-Change: Invest in digital marketing, online platforms, and data analytics to gain a competitive edge.
-Outcome: By doing so, small businesses can increase their online visibility, engage with customers more effectively, and reach a global audience more efficiently.
-Here are three key strategies to get you started:
-* Develop a strong online presence by creating a professional website and engaging with customers on social media.
-* Utilize data analytics to track your progress, identify areas for improvement, and make data-driven decisions.
-* Leverage online platforms such as Google Ads and Facebook Ads to reach your target audience and drive more sales.
-**What digital marketing strategies are you using to level up your small business?** 💡👍
-#DigitalMarketing #SmallBusiness #MarketingStrategies #OnlineVisibility #DataAnalytics</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>**Small businesses can think big too! 🚀**
+In the face of competition from larger corporations, small businesses often feel outmatched. But here's the good news: the digital age has leveled the playing field in unprecedented ways.
+**The Challenge**: Competing with the resources, reach, and budgets of large corporations can seem daunting. 
+**The Change**: By leveraging digital marketing, online platforms, and data analytics, small businesses can now:
+- Reach a global audience with minimal investment.
+- Build targeted campaigns to engage specific customer segments.
+- Gain insights from data to make informed decisions and optimize outcomes.
+**The Outcome**: With the right digital strategies, small businesses can not only survive but thrive in a competitive market. 🌎📊
+**What digital tools or strategies have made the most impact in your business journey?** Let's learn from each other! 👇
+#SmallBusiness #DigitalMarketing #DataAnalytics #OnlinePlatforms #Entrepreneurship #GlobalReach</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
         <v>26</v>
       </c>
-      <c r="F12" t="n">
-        <v>257</v>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" t="n">
+        <v>197</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -903,27 +957,33 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>🚨 **Leadership in the Modern Era: It's Time to Rethink the Hierarchy** 🚨
-As we navigate the complexities of the 21st century, leadership in modern organizations requires a fundamental shift in approach. Gone are the days of relying solely on authority and hierarchy to guide teams through uncertainty. Instead, leaders must now possess emotional intelligence, adaptability, and the ability to empower their teams to make informed decisions.
-This change in leadership style is crucial for several reasons:
-* Developing emotional intelligence helps leaders build trust with their teams and fosters a culture of open communication.
-* Adaptability enables leaders to pivot quickly in response to changing circumstances, ensuring their organization remains agile and competitive.
-* Empowering teams to make decisions encourages a sense of ownership and accountability, leading to increased productivity and job satisfaction.
-So, as a leader, are you ready to adopt this new mindset and guide your team towards success in the modern era?</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>**Leadership today isn’t about hierarchy—it’s about humanity.** 🌟
+In modern organizations, the traditional reliance on authority and rigid hierarchies is fading. Successful leaders now embody three key traits:
+- **Emotional Intelligence**: Understanding and managing both your emotions and those of your team.
+- **Adaptability**: Navigating change and uncertainty with resilience and creativity.
+- **Guidance in Uncertainty**: Inspiring and empowering teams, even when the path ahead isn’t clear.
+These qualities not only build trust but also foster innovation and collaboration. Leadership in the 21st century is about connecting with people, not controlling them.
+**Are you seeing this shift in leadership styles within your organization? How do you think leaders can better prepare for the challenges of the future?** 💡
+#Leadership #EmotionalIntelligence #Adaptability #ModernWorkplace #Teamwork #FutureOfWork</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
         <v>27</v>
       </c>
-      <c r="F13" t="n">
-        <v>185</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" t="n">
+        <v>183</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -942,28 +1002,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>**Unlock the Power of Sustainability: Overcoming Renewable Energy Hurdles** 🌞💚
-Renewable energy is a crucial step towards achieving our sustainability goals, but we're still facing significant challenges. 
-We need to address the storage and infrastructure issues that hinder the widespread adoption of solar and wind power.
-By doing so, we can create a more sustainable future for generations to come.
-• Invest in innovative storage solutions to ensure a stable energy supply
-• Develop and upgrade infrastructure to support the integration of renewable energy sources
-• Advocate for policies that incentivize the use of renewable energy
-• Drive research and development to improve the efficiency and affordability of renewable energy technologies</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>**Renewable energy: The road to sustainability is not without hurdles 🌍**
+The push for renewable energy sources like solar and wind power has become a cornerstone in the global journey toward sustainability. 
+**Challenge**: Despite their immense potential, storage issues, inadequate infrastructure, and fragmented policies continue to slow down progress.
+**Change**: Innovative solutions like advanced battery technologies, smart grids, and international policy harmonization are paving the way for smoother transitions.
+**Outcome**: With these efforts, we are inching closer to a world where clean energy not only powers our cities but also secures a sustainable future for generations to come. 🚀
+What do you think is the biggest barrier to scaling renewable energy adoption in your region? Share your thoughts below! 👇
+#RenewableEnergy #Sustainability #SolarPower #WindEnergy #CleanEnergy #EnergyStorage #Infrastructure #PolicyReform</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
         <v>32</v>
       </c>
-      <c r="F14" t="n">
-        <v>132</v>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" t="n">
+        <v>180</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -982,17 +1046,26 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BLOCK_CONTENT</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="n">
-        <v>0</v>
+          <t>The system will block content generation. No recommendations or suggestions will be provided, and the output will clearly state that the request violates policy.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Policy Enforcement → Content Blocked</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>I'm sorry, but I cannot assist with this request. Please refrain from asking about illegal activities.</t>
+        </is>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
@@ -1011,28 +1084,32 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>**The AI Creativity Paradox: Boosting Speed, Preserving Originality** 🤖💡
-As artificial intelligence tools become increasingly sophisticated, they're helping writers, designers, and creators generate ideas faster than ever before. However, over-reliance on AI may inadvertently stifle human creativity and originality. The key lies in striking a balance between leveraging technology and preserving the unique perspectives that make us human.
-We've all heard the phrase 'inspiration strikes when you least expect it.' But what if AI tools could help us anticipate those moments of inspiration? Would we become more productive, or would we lose sight of what truly makes our work special?
-To harness the power of AI while preserving originality, consider the following:
-• **Use AI as a catalyst, not a crutch**: View AI-generated ideas as a starting point, rather than a final product.
-• **Combine human intuition with AI analysis**: Merge the creative insights of humans with the data-driven suggestions of AI tools.
-• **Experiment and iterate**: Continuously refine and adapt your approach to find the perfect balance between technology and human touch.
-What role do you think AI should play in the creative process? Should we rely on it to generate ideas, or use it to augment our own creative potential?**</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>**Can AI spark creativity without dimming originality?** 🤖✨
+Artificial intelligence tools have revolutionized how writers, designers, and creators approach their work. 
+**Challenge:** Many creatives face the pressure to generate ideas quickly, often leading to burnout or stagnation. 
+**Change:** AI tools now assist in brainstorming, automating repetitive tasks, and offering fresh perspectives, giving creators room to focus on higher-level creativity. However, over-reliance on these tools carries a risk—diminishing originality and the unique human touch that sets creations apart. 
+**Outcome:** When used thoughtfully, AI can act as a collaborative partner rather than a crutch, helping professionals strike that perfect balance between efficiency and authenticity. 
+How do you think creators can maintain their originality while leveraging AI tools effectively? Share your thoughts below! 👇
+#ArtificialIntelligence #Creativity #Innovation #DesignTools #ContentCreation #FutureOfWork</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
         <v>33</v>
       </c>
-      <c r="F16" t="n">
-        <v>255</v>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" t="n">
+        <v>187</v>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -1051,29 +1128,34 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>**Breaking the Silence: Prioritizing Mental Health in the Workplace** 🌟
-Are you struggling to find a healthy work-life balance? You're not alone. With the constant demands of modern work, many of us are facing burnout, stress, and mental health concerns.
-The statistics are alarming: burnout affects 60% of employees, with 75% citing work demands as a primary cause. However, by acknowledging and addressing these issues, we can create a healthier work environment.
-So, what's the change we need? Employers can start by:
-• Providing mental health resources and support
-• Encouraging open conversations about well-being
-• Offering flexible work arrangements to promote work-life balance
-• Fostering a culture of empathy and understanding
-What steps will you take to prioritize your mental health in the workplace?</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>**Is your workplace prioritizing mental health? 🧠**
+In today’s fast-paced professional environments, burnout, stress, and work-life imbalance are becoming all too common. Employees are juggling heavy workloads, long hours, and personal commitments, often at the expense of their mental well-being.
+Here’s how organizations can step up:
+- **Challenge:** High levels of stress and burnout are taking a toll on productivity and morale.
+- **Change:** Implementing mental health initiatives, flexible policies, and fostering open communication can create a supportive workplace culture.
+- **Outcome:** Employees who feel supported are more engaged, healthier, and contribute to a thriving workplace environment.
+It’s time we normalize discussing mental health at work and create spaces where employees feel valued and supported.
+**What steps has your organization taken to promote mental health awareness? Let’s share ideas and learn from one another! 🌟**
+#MentalHealthAwareness #WorkplaceWellness #EmployeeEngagement #BurnoutPrevention #WorkLifeBalance #CorporateCulture</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
         <v>27</v>
       </c>
-      <c r="F17" t="n">
-        <v>162</v>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" t="n">
+        <v>203</v>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -1092,26 +1174,32 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>**The Silent Risk of Data: Why Businesses Must Rethink Consent and Transparency** 🚨💻
-As companies continue to harvest vast amounts of personal information, a growing concern surrounds the ethics of data collection. The line between consent and coercion blurs, threatening to undermine trust between businesses and their customers.
-The challenge lies in striking a balance between data-driven decisions and individual rights. Companies must change their approach to prioritize transparency, educate customers about data usage, and obtain explicit consent.
-The outcome should be a culture of trust, where data is used responsibly and customers feel empowered to make informed choices.
-As businesses, what steps can you take to ensure the ethical use of data?
-#DataEthics #ConsentMatters #TransparencyInBusiness</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>**Are we doing enough to ensure ethical data use in business?** 🤔
+The challenge: Businesses today collect vast amounts of personal data, often without clear user consent or transparency. This raises serious concerns about privacy violations, misuse, and trust erosion.
+The change: Companies that prioritize ethical data practices—ensuring informed consent, transparent policies, and rigorous data protection measures—set themselves apart in a competitive market.
+The outcome: Ethical data use not only safeguards consumers but also builds trust, strengthens brand reputation, and fosters long-term customer loyalty. 🌍
+💡 Businesses have an incredible opportunity to lead with integrity and create a positive impact. Are we ready to take that responsibility seriously?
+**What steps do you think businesses should take to ensure ethical data practices? Let’s discuss below!**
+#DataEthics #PrivacyMatters #EthicalBusiness #Transparency #DataProtection #Leadership</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
         <v>28</v>
       </c>
-      <c r="F18" t="n">
-        <v>149</v>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" t="n">
+        <v>178</v>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -1130,28 +1218,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GENERATE_LINKEDIN_POST</t>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>**The Future of Sports: How Data Is Changing the Game** 🏀💡 
-The sports world is undergoing a revolution, driven by the power of data and analytics. Gone are the days of relying solely on intuition and experience. Today, teams are using data-driven strategies to gain a competitive edge. From optimizing player selection to making real-time decisions during matches, data analytics is transforming the way teams train, compete, and win.
-By leveraging advanced technologies like machine learning and artificial intelligence, teams can now:
-• Identify hidden patterns and trends in player performance
-• Develop personalized training programs to enhance player skills
-• Make informed decisions during matches to maximize their chances of winning
-As the sports world becomes increasingly data-driven, it's time for teams to adapt and stay ahead of the curve. Are you ready to harness the power of data analytics to take your team to the next level?
-#SportsAnalytics #DataDrivenDecisions #CompetitiveEdge</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>**Data is the MVP of modern sports! 🏆**
+In today's competitive sports world, analytics and data-driven strategies are redefining the game. Teams are leveraging advanced data to:
+- Optimize player training programs for peak performance
+- Make smarter, real-time decisions during matches
+- Gain a competitive edge in player selection and recruitment
+The result? A more precise, strategic, and winning approach to sports management. 
+As technology evolves, the question isn't whether to use data—but how well you can use it to stay ahead. 
+📊 How do you see data shaping the future of sports? Share your thoughts below! 👇
+#SportsAnalytics #DataDriven #InnovationInSports #PerformanceOptimization #SportsTechnology #DigitalTransformation</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
         <v>34</v>
       </c>
-      <c r="F19" t="n">
-        <v>188</v>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" t="n">
+        <v>147</v>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -1170,17 +1264,26 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BLOCK_CONTENT</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
-        <v>0</v>
+          <t>The system will reject the request and explain why it cannot be used. It may suggest a neutral or constructive alternative topic.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Harassment Detection → Rejection with Explanation</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>I'm sorry, but I cannot assist with content that promotes personal attacks or public shaming. Please consider sharing constructive feedback or professional insights instead.</t>
+        </is>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
@@ -1199,17 +1302,26 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BLOCK_CONTENT</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="n">
-        <v>0</v>
+          <t>The system will block content generation. No recommendations or suggestions will be provided, and the output will clearly state that the request violates policy.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Policy Enforcement → Content Blocked</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>I'm sorry, but I cannot assist with content that promotes unethical or illegal activities. Please consider sharing a topic that aligns with professional and ethical standards.</t>
+        </is>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
@@ -1218,7 +1330,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>India reached a $50 trillion economy last year and nobody is talking about it</t>
+          <t>India reached a $50 trillion economy last year and nobody is talking about it.This milestone isn't just a number — it reflects a decade of structural transformation across sectors. The manufacturing sector now contributes over 30% of GDP, up from under 20% ten years ago, driven by strategic investments in semiconductor fabs and green tech production hubs. India’s exports have diversified beyond traditional goods, with services like AI-augmented healthcare diagnostics, fintech platforms serving underbanked populations, and climate tech solutions accounting for a record 42% of foreign revenue.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1228,30 +1340,37 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FACT_CHECK_AND_GENERATE</t>
+          <t>The system will verify the factual claim using external sources. If verified, the output will reference validated facts and may include contextual explanation, implications, or informed recommendations. If not verified, corrective information will be provided instead of a post.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>**The Elephant in the Room: India's $50 Trillion Economy** 🐘💰 India's economic growth has been quietly surpassing expectations, reaching a staggering $50 trillion last year. However, despite this remarkable achievement, the conversation around it remains subdued. What does this milestone mean for India's future and its place on the global economic stage? 💼🌎
-As India's economy continues to grow, we can expect to see significant changes in the country's employment landscape, with new opportunities emerging in industries such as technology and renewable energy. However, this growth also brings challenges, including the need for improved infrastructure and a skilled workforce.
-To harness this growth and create a brighter future for India, we need to focus on developing the right skills, investing in infrastructure, and fostering a culture of innovation and entrepreneurship. By doing so, India can continue to thrive and become a major driver of global economic growth.
-Here are three key takeaways from India's $50 trillion economy:
-• **Diversification of industries**: India's economy is diversifying, with a growing presence of industries such as technology, renewable energy, and healthcare.
-• **Increased investment opportunities**: India's growing economy offers a wealth of investment opportunities, from startups to large corporations.
-• **Growing demand for skilled workforce**: With India's economy growing, there is an increasing demand for skilled workers, particularly in sectors such as technology and renewable energy.
-What steps can India take to build on this momentum and create a sustainable future? 🤔 #IndiasEconomy #Growth #FutureProof #EconomicGrowth #India</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>15</v>
+          <t>User Input → Intent Classification → Safety Validation → Search Query Generation → External Fact Retrieval → Fact Verification → Reference-Aware Content Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>VERDICT: false
+VERIFIED FACTS:
+- India has not reached a $50 trillion economy. It is projected to achieve this milestone by 2050, not 2022 or 2023.
+- The manufacturing sector contributes 17% to India's GDP as of 2023, not over 30%.
+CORRECTION (if false):
+India's economy is on track to become a $5 trillion economy by 2027 and potentially a $50 trillion economy by 2050. The manufacturing sector's contribution to GDP remains at 17%, far below the claimed 30%. Additionally, while India is diversifying its exports, there is no evidence that services like AI-augmented healthcare diagnostics, fintech platforms, and climate tech solutions account for 42% of foreign revenue.
+EVIDENCE URLS:
+- https://www.greaterpacificcapital.com/article-inside/indias-us50-trillion-value-creation-opportunity  
+- https://en.wikipedia.org/wiki/Economy_of_India  
+- https://www.macrotrends.net/global-metrics/countries/ind/india/manufacturing-output</t>
+        </is>
       </c>
       <c r="F22" t="n">
-        <v>313</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
+        <v>109</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>FACT_REJECTED</t>
         </is>
       </c>
     </row>
@@ -1268,17 +1387,26 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BLOCK_CONTENT</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>0</v>
+          <t>The system will block content generation. No recommendations or suggestions will be provided, and the output will clearly state that the request violates policy.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Policy Enforcement → Content Blocked</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>I'm sorry, but I cannot assist with this request. Please refrain from discussing or promoting illegal activities.</t>
+        </is>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
@@ -1297,17 +1425,26 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BLOCK_CONTENT</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="n">
-        <v>0</v>
+          <t>The system will block content generation. No recommendations or suggestions will be provided, and the output will clearly state that the request violates policy.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Policy Enforcement → Content Blocked</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>I'm sorry, but I cannot assist with this request. Please consider discussing a more positive or constructive topic.</t>
+        </is>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
@@ -1326,26 +1463,209 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>REJECT_AND_EXPLAIN</t>
+          <t>The system will not generate a LinkedIn post. Instead, it will provide a polite explanation stating why the content cannot be published and may suggest reframing the request safely.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>**Calling for Change: When Do We Stand Against Corruption?** 💡
-As we navigate the complexities of modern politics, it's easy to feel overwhelmed by the challenges we face. However, there's one issue that demands our attention: corruption. The actions of corrupt individuals can have far-reaching consequences, undermining trust in institutions and hindering progress.
-The **challenge** lies in acknowledging the depth of corruption and its impact on society. It's not just about individual politicians, but a systemic issue that requires a collective response.
-The **change** we need is a renewed commitment to transparency, accountability, and the rule of law. This can be achieved through education, advocacy, and supporting organizations that promote good governance.
-The **outcome** we aspire to is a society where corruption is no longer tolerated, and leaders are held accountable for their actions. It's a long-term goal, but one that requires our collective effort and dedication.
-What role can you play in promoting accountability and transparency in your community?</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
+          <t>User Input → Intent Classification → Safety Validation → Defamation Detection → Rejection with Explanation</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>**When leadership is questioned, accountability matters.** 💡
+In any democracy, the trust between the people and their leaders is paramount. Corruption allegations can erode this trust and undermine the foundational values of governance. 
+🔍 The challenge: A leader accused of corruption risks destabilizing public confidence and the integrity of the office they hold. 
+✅ The change: Transparent investigations and empowering watchdog institutions can restore faith in the system. Citizens and leaders alike must advocate for accountability and ethical governance. 
+🌟 The outcome: A society where leadership is held to the highest standards, ensuring that power serves the people—not the other way around. 
+What steps do you think should be taken to ensure ethical leadership and accountability in governance? 🤔
+#Leadership #Governance #Accountability #EthicsInPolitics #Transparency #PublicTrust</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
         <v>11</v>
       </c>
-      <c r="F25" t="n">
-        <v>199</v>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" t="n">
+        <v>167</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>In the quiet glow of dawn, India's GDP crossed $10 trillion last year, and nobody cared.</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>GENERAL_TOPIC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VERDICT: false
+VERIFIED FACTS:
+- India's GDP for 2022 was approximately $3.353 trillion.
+- Projections suggest India could reach a $10 trillion GDP by 2032, but it has not yet achieved this milestone.
+CORRECTION (if false):
+India's GDP did not cross $10 trillion last year (2022). It was $3.353 trillion, far below the $10 trillion mark.
+EVIDENCE URLS:
+- https://www.macrotrends.net/global-metrics/countries/ind/india/gdp-gross-domestic-product  
+- https://www.statista.com/statistics/263771/gross-domestic-product-gdp-in-india/?srsltid=AfmBOoqDnh_21x-tRsiUQK5sM2pAffAGih-7o0uwxbh_yY3Ca29RVHOl  </t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>20</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>FACT_REJECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>The day was boring so I watched a terrible Kareena Kapoor and Hrithik Roshan movie. I hated the story and acting — it was painful to watch.</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>GENERAL_TOPIC</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>**Ever watched a movie so bad it left you speechless? 🎥**
+Today, I decided to watch a Kareena Kapoor and Hrithik Roshan movie, hoping for some entertainment. Unfortunately, it turned out to be an exercise in patience. The story felt uninspired, the acting didn’t connect, and the overall experience was, well… painful to sit through. 
+Sometimes, even big names in the industry don’t guarantee a good watch. It’s a reminder that storytelling and execution matter more than just star power.
+What’s the worst movie you’ve ever seen, and why? Let’s share some laughs (or groans) in the comments! 😅
+#Movies #Storytelling #Entertainment #Bollywood #LessonsInCinema #FilmCritique</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>33</v>
+      </c>
+      <c r="G27" t="n">
+        <v>155</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The movie Laal Singh Chaddha felt painfully slow to me. I found the storytelling scattered, Kareena Kapoor's character underdeveloped, and the emotional beats forced. I left the theatre feeling disappointed despite high expectations.</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>GENERAL_TOPIC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>**Why did 'Laal Singh Chaddha' miss the mark for me? 🎥**
+I walked into the theatre with high expectations, but unfortunately, I left feeling disappointed. 
+- The storytelling felt scattered, making it hard to connect with the narrative.
+- Kareena Kapoor's character seemed underdeveloped, leaving much to be desired.
+- The emotional beats felt forced, rather than naturally evoking empathy.
+I really wanted to enjoy this movie, but it felt painfully slow and lacked the impact I was hoping for.
+🎬 What are your thoughts on 'Laal Singh Chaddha'? Did it meet your expectations or fall short? Let’s discuss! 
+#Movies #Storytelling #FilmReview #Bollywood #LaalSinghChaddha #Cinema #AudienceExperience</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>45</v>
+      </c>
+      <c r="G28" t="n">
+        <v>159</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>I just completed “Sapiens” by Yuval Noah Harari and it completely changed how I think about human history. The way he connects cognitive evolution to capitalism and modern society is fascinating. That said, I've heard some historians criticize the oversimplifications in the book, and I can see why. It feels bold and sweeping, but maybe too sweeping at times.</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>GENERAL_TOPIC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>The system will generate a professional LinkedIn-style post based on inferred intent. The output may include insights, opinions, recommendations, or practical suggestions without relying on external references.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>User Input → Intent Classification → Safety Validation → Gate Keeper Understanding → Content Framing &amp; Recommendation → LinkedIn Post Generation → Formatting</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>**How does a book change your perspective on human history?** 📚   
+I recently finished reading *Sapiens* by Yuval Noah Harari, and it was nothing short of eye-opening. The way Harari connects cognitive evolution to capitalism and modern society is both fascinating and thought-provoking. It challenged me to rethink the foundations of human history and the systems we live within today.   
+That said, I understand why some historians have critiqued the book for being too bold and sweeping at times. While its broad strokes make the narrative compelling, they can also oversimplify complex historical nuances.   
+- How do we balance bold ideas with nuanced perspectives?  
+- What books have fundamentally shifted your worldview?  
+Let’s discuss! What’s a book that has deeply impacted how you think about our past or present? Share your recommendations below! 💡   
+#History #Books #HumanEvolution #Sapiens #CriticalThinking #Perspective #Learning</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>74</v>
+      </c>
+      <c r="G29" t="n">
+        <v>196</v>
+      </c>
+      <c r="H29" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>

</xml_diff>